<commit_message>
fix(video): preenche seguidores que a planilha da demo deixava em branco
YouTube veio do IP local. Instagram e TikTok estavam bloqueados nesse IP, então as contagens saíram das APIs que o Radar já usa.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/metricas/chatguru/metricas-concorrentes-chatguru.xlsx
+++ b/outputs/metricas/chatguru/metricas-concorrentes-chatguru.xlsx
@@ -1093,14 +1093,20 @@
         <v>116000</v>
       </c>
       <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
+      <c r="P2" s="3" t="n">
+        <v>1062</v>
+      </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>https://www.instagram.com/BlipBR/</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@blipbr</t>
+        </is>
+      </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>https://www.blip.ai/blog/whatsapp/atendimento-via-whatsapp/</t>
@@ -1311,7 +1317,9 @@
           <t>https://www.linkedin.com/ad-library/search?payer=Total+Chat</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="n">
+        <v>10844</v>
+      </c>
       <c r="O5" s="8" t="n">
         <v>2029</v>
       </c>
@@ -1381,7 +1389,9 @@
           <t>https://www.linkedin.com/ad-library/search?payer=Multiatendimento+WhatsApp</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="n">
+        <v>36</v>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="inlineStr">

</xml_diff>